<commit_message>
Curva S actualizada 2026-07-05 14:33 Chile
</commit_message>
<xml_diff>
--- a/data/50001566 - XEMORTIZ.xlsx
+++ b/data/50001566 - XEMORTIZ.xlsx
@@ -3805,7 +3805,7 @@
         <v>46198.51051443287</v>
       </c>
       <c r="D41" s="8">
-        <v>46198.510531990745</v>
+        <v>46208.70532195602</v>
       </c>
       <c r="E41" s="9" t="s">
         <v>153</v>
@@ -3847,7 +3847,7 @@
         <v>46213</v>
       </c>
       <c r="R41" s="8">
-        <v>46190</v>
+        <v>46220</v>
       </c>
       <c r="S41" s="11" t="s">
         <v>77</v>

</xml_diff>

<commit_message>
Curva S actualizada 2026-08-29 18:43 Chile
</commit_message>
<xml_diff>
--- a/data/50001566 - XEMORTIZ.xlsx
+++ b/data/50001566 - XEMORTIZ.xlsx
@@ -1646,7 +1646,7 @@
         <v>46197.84318319445</v>
       </c>
       <c r="D4" s="5">
-        <v>46197.8432930787</v>
+        <v>46263.77739836805</v>
       </c>
       <c r="E4" s="6" t="s">
         <v>24</v>
@@ -1947,7 +1947,7 @@
         <v>46197.84431706018</v>
       </c>
       <c r="D9" s="8">
-        <v>46197.84432748843</v>
+        <v>46263.76700403936</v>
       </c>
       <c r="E9" s="9" t="s">
         <v>44</v>
@@ -2951,7 +2951,7 @@
         <v>46224.832077025465</v>
       </c>
       <c r="D25" s="8">
-        <v>46224.83209384259</v>
+        <v>46263.76745226852</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>99</v>
@@ -4011,7 +4011,7 @@
       </c>
       <c r="C43" s="9"/>
       <c r="D43" s="8">
-        <v>46262.18089949074</v>
+        <v>46263.76860283565</v>
       </c>
       <c r="E43" s="9" t="s">
         <v>160</v>
@@ -4650,7 +4650,7 @@
         <v>46260.58671038195</v>
       </c>
       <c r="D54" s="5">
-        <v>46260.59069322917</v>
+        <v>46263.76957377315</v>
       </c>
       <c r="E54" s="6" t="s">
         <v>194</v>
@@ -4825,7 +4825,7 @@
         <v>46260.5869990625</v>
       </c>
       <c r="D57" s="8">
-        <v>46260.58701207176</v>
+        <v>46263.76959292824</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>205</v>
@@ -4998,7 +4998,7 @@
       </c>
       <c r="C60" s="6"/>
       <c r="D60" s="5">
-        <v>46260.59071152778</v>
+        <v>46263.76967357639</v>
       </c>
       <c r="E60" s="6" t="s">
         <v>213</v>
@@ -5513,7 +5513,7 @@
       </c>
       <c r="C69" s="9"/>
       <c r="D69" s="8">
-        <v>46263.17081568287</v>
+        <v>46263.77353957176</v>
       </c>
       <c r="E69" s="9" t="s">
         <v>235</v>
@@ -5682,7 +5682,7 @@
       </c>
       <c r="C72" s="6"/>
       <c r="D72" s="5">
-        <v>46258.19795055556</v>
+        <v>46263.77368297454</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>241</v>
@@ -5851,7 +5851,7 @@
       </c>
       <c r="C75" s="9"/>
       <c r="D75" s="8">
-        <v>46260.59090943287</v>
+        <v>46263.77374159722</v>
       </c>
       <c r="E75" s="9" t="s">
         <v>247</v>
@@ -6014,7 +6014,7 @@
       </c>
       <c r="C78" s="6"/>
       <c r="D78" s="5">
-        <v>46260.59092870371</v>
+        <v>46263.77409542824</v>
       </c>
       <c r="E78" s="6" t="s">
         <v>252</v>
@@ -6181,7 +6181,7 @@
       </c>
       <c r="C81" s="9"/>
       <c r="D81" s="8">
-        <v>46261.20224831019</v>
+        <v>46263.77417350694</v>
       </c>
       <c r="E81" s="9" t="s">
         <v>258</v>
@@ -6348,7 +6348,7 @@
       </c>
       <c r="C84" s="6"/>
       <c r="D84" s="5">
-        <v>46260.59096447917</v>
+        <v>46263.77543009259</v>
       </c>
       <c r="E84" s="6" t="s">
         <v>263</v>
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C88" s="6"/>
       <c r="D88" s="5">
-        <v>46195.58618233797</v>
+        <v>46263.77570484954</v>
       </c>
       <c r="E88" s="6" t="s">
         <v>272</v>
@@ -6731,7 +6731,7 @@
       </c>
       <c r="C91" s="9"/>
       <c r="D91" s="8">
-        <v>46260.591004409725</v>
+        <v>46263.77620959491</v>
       </c>
       <c r="E91" s="9" t="s">
         <v>280</v>
@@ -6900,7 +6900,7 @@
       </c>
       <c r="C94" s="6"/>
       <c r="D94" s="5">
-        <v>46260.59102431713</v>
+        <v>46263.77653796296</v>
       </c>
       <c r="E94" s="6" t="s">
         <v>285</v>
@@ -7065,7 +7065,7 @@
       </c>
       <c r="C97" s="9"/>
       <c r="D97" s="8">
-        <v>46195.5866459838</v>
+        <v>46263.77670127315</v>
       </c>
       <c r="E97" s="9" t="s">
         <v>291</v>

</xml_diff>